<commit_message>
Dashboard: 2026-07-09 17:36 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1027,11 +1027,11 @@
         <v>7</v>
       </c>
       <c r="E32" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -1593,11 +1593,11 @@
         <v>7</v>
       </c>
       <c r="E63" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -2159,11 +2159,11 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -3857,11 +3857,11 @@
         <v>7</v>
       </c>
       <c r="E187" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4427,7 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -4993,7 +4993,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -5559,7 +5559,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -6125,7 +6125,7 @@
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -6687,11 +6687,11 @@
         <v>7</v>
       </c>
       <c r="E342" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -7253,11 +7253,11 @@
         <v>7</v>
       </c>
       <c r="E373" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -7819,11 +7819,11 @@
         <v>7</v>
       </c>
       <c r="E404" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -8389,7 +8389,7 @@
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -8955,7 +8955,7 @@
       </c>
       <c r="F466" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -9517,11 +9517,11 @@
         <v>7</v>
       </c>
       <c r="E497" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F497" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -10087,7 +10087,7 @@
       </c>
       <c r="F528" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -10649,11 +10649,11 @@
         <v>7</v>
       </c>
       <c r="E559" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F559" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -11219,7 +11219,7 @@
       </c>
       <c r="F590" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -11781,11 +11781,11 @@
         <v>7</v>
       </c>
       <c r="E621" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F621" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -12347,11 +12347,11 @@
         <v>7</v>
       </c>
       <c r="E652" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F652" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -12917,7 +12917,7 @@
       </c>
       <c r="F683" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -13479,11 +13479,11 @@
         <v>7</v>
       </c>
       <c r="E714" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F714" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -14049,7 +14049,7 @@
       </c>
       <c r="F745" t="inlineStr">
         <is>
-          <t>2026-07-09 11:50</t>
+          <t>2026-07-09 14:33</t>
         </is>
       </c>
     </row>
@@ -14360,7 +14360,7 @@
         <v>0</v>
       </c>
       <c r="AF2" t="n">
-        <v>353</v>
+        <v>357</v>
       </c>
     </row>
     <row r="3">
@@ -14460,7 +14460,7 @@
         <v>0</v>
       </c>
       <c r="AF3" t="n">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="4">
@@ -14560,7 +14560,7 @@
         <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5">
@@ -14660,7 +14660,7 @@
         <v>0</v>
       </c>
       <c r="AF5" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6">
@@ -14760,7 +14760,7 @@
         <v>2818</v>
       </c>
       <c r="AF6" t="n">
-        <v>963</v>
+        <v>981</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-07-14 15:19 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1027,11 +1027,11 @@
         <v>7</v>
       </c>
       <c r="E32" t="n">
-        <v>103</v>
+        <v>121</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -1593,11 +1593,11 @@
         <v>7</v>
       </c>
       <c r="E63" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -2159,11 +2159,11 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -3291,11 +3291,11 @@
         <v>7</v>
       </c>
       <c r="E156" t="n">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -3857,11 +3857,11 @@
         <v>7</v>
       </c>
       <c r="E187" t="n">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -4423,11 +4423,11 @@
         <v>7</v>
       </c>
       <c r="E218" t="n">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -4989,11 +4989,11 @@
         <v>7</v>
       </c>
       <c r="E249" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -5555,11 +5555,11 @@
         <v>7</v>
       </c>
       <c r="E280" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -6121,11 +6121,11 @@
         <v>7</v>
       </c>
       <c r="E311" t="n">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -6687,11 +6687,11 @@
         <v>7</v>
       </c>
       <c r="E342" t="n">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -7253,11 +7253,11 @@
         <v>7</v>
       </c>
       <c r="E373" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -7819,11 +7819,11 @@
         <v>7</v>
       </c>
       <c r="E404" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -8385,11 +8385,11 @@
         <v>7</v>
       </c>
       <c r="E435" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -8951,11 +8951,11 @@
         <v>7</v>
       </c>
       <c r="E466" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F466" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -9517,11 +9517,11 @@
         <v>7</v>
       </c>
       <c r="E497" t="n">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="F497" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -10083,11 +10083,11 @@
         <v>7</v>
       </c>
       <c r="E528" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F528" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -10649,11 +10649,11 @@
         <v>7</v>
       </c>
       <c r="E559" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="F559" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -11215,11 +11215,11 @@
         <v>7</v>
       </c>
       <c r="E590" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F590" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -11781,11 +11781,11 @@
         <v>7</v>
       </c>
       <c r="E621" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="F621" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -12347,11 +12347,11 @@
         <v>7</v>
       </c>
       <c r="E652" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F652" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -12913,11 +12913,11 @@
         <v>7</v>
       </c>
       <c r="E683" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F683" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -13479,11 +13479,11 @@
         <v>7</v>
       </c>
       <c r="E714" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="F714" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -14045,11 +14045,11 @@
         <v>7</v>
       </c>
       <c r="E745" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F745" t="inlineStr">
         <is>
-          <t>2026-07-13 14:37</t>
+          <t>2026-07-14 12:16</t>
         </is>
       </c>
     </row>
@@ -14360,7 +14360,7 @@
         <v>0</v>
       </c>
       <c r="AF2" t="n">
-        <v>481</v>
+        <v>520</v>
       </c>
     </row>
     <row r="3">
@@ -14460,7 +14460,7 @@
         <v>0</v>
       </c>
       <c r="AF3" t="n">
-        <v>489</v>
+        <v>546</v>
       </c>
     </row>
     <row r="4">
@@ -14560,7 +14560,7 @@
         <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>320</v>
+        <v>376</v>
       </c>
     </row>
     <row r="5">
@@ -14660,7 +14660,7 @@
         <v>0</v>
       </c>
       <c r="AF5" t="n">
-        <v>105</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6">
@@ -14760,7 +14760,7 @@
         <v>2818</v>
       </c>
       <c r="AF6" t="n">
-        <v>1395</v>
+        <v>1559</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-07-22 15:58 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1027,11 +1027,11 @@
         <v>7</v>
       </c>
       <c r="E32" t="n">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -1593,11 +1593,11 @@
         <v>7</v>
       </c>
       <c r="E63" t="n">
-        <v>205</v>
+        <v>225</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -2159,11 +2159,11 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -3291,11 +3291,11 @@
         <v>7</v>
       </c>
       <c r="E156" t="n">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -3857,11 +3857,11 @@
         <v>7</v>
       </c>
       <c r="E187" t="n">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -4423,11 +4423,11 @@
         <v>7</v>
       </c>
       <c r="E218" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -4989,11 +4989,11 @@
         <v>7</v>
       </c>
       <c r="E249" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -5555,11 +5555,11 @@
         <v>7</v>
       </c>
       <c r="E280" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -6121,11 +6121,11 @@
         <v>7</v>
       </c>
       <c r="E311" t="n">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -6687,11 +6687,11 @@
         <v>7</v>
       </c>
       <c r="E342" t="n">
-        <v>181</v>
+        <v>201</v>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -7253,11 +7253,11 @@
         <v>7</v>
       </c>
       <c r="E373" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -7819,11 +7819,11 @@
         <v>7</v>
       </c>
       <c r="E404" t="n">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -8385,11 +8385,11 @@
         <v>7</v>
       </c>
       <c r="E435" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -8951,11 +8951,11 @@
         <v>7</v>
       </c>
       <c r="E466" t="n">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="F466" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -9517,11 +9517,11 @@
         <v>7</v>
       </c>
       <c r="E497" t="n">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="F497" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -10083,11 +10083,11 @@
         <v>7</v>
       </c>
       <c r="E528" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F528" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -10649,11 +10649,11 @@
         <v>7</v>
       </c>
       <c r="E559" t="n">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="F559" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -11215,11 +11215,11 @@
         <v>7</v>
       </c>
       <c r="E590" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F590" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -11781,11 +11781,11 @@
         <v>7</v>
       </c>
       <c r="E621" t="n">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="F621" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -12347,11 +12347,11 @@
         <v>7</v>
       </c>
       <c r="E652" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="F652" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -12913,11 +12913,11 @@
         <v>7</v>
       </c>
       <c r="E683" t="n">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="F683" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -13479,11 +13479,11 @@
         <v>7</v>
       </c>
       <c r="E714" t="n">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="F714" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -14049,7 +14049,7 @@
       </c>
       <c r="F745" t="inlineStr">
         <is>
-          <t>2026-07-21 12:58</t>
+          <t>2026-07-22 12:54</t>
         </is>
       </c>
     </row>
@@ -14360,7 +14360,7 @@
         <v>0</v>
       </c>
       <c r="AF2" t="n">
-        <v>809</v>
+        <v>850</v>
       </c>
     </row>
     <row r="3">
@@ -14460,7 +14460,7 @@
         <v>0</v>
       </c>
       <c r="AF3" t="n">
-        <v>849</v>
+        <v>909</v>
       </c>
     </row>
     <row r="4">
@@ -14560,7 +14560,7 @@
         <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>589</v>
+        <v>624</v>
       </c>
     </row>
     <row r="5">
@@ -14660,7 +14660,7 @@
         <v>0</v>
       </c>
       <c r="AF5" t="n">
-        <v>378</v>
+        <v>418</v>
       </c>
     </row>
     <row r="6">
@@ -14760,7 +14760,7 @@
         <v>2818</v>
       </c>
       <c r="AF6" t="n">
-        <v>2625</v>
+        <v>2801</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-08-12 10:55 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1045,11 +1045,11 @@
         <v>8</v>
       </c>
       <c r="E33" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -1629,11 +1629,11 @@
         <v>8</v>
       </c>
       <c r="E65" t="n">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -2213,11 +2213,11 @@
         <v>8</v>
       </c>
       <c r="E97" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -3381,11 +3381,11 @@
         <v>8</v>
       </c>
       <c r="E161" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -3965,11 +3965,11 @@
         <v>8</v>
       </c>
       <c r="E193" t="n">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -4549,11 +4549,11 @@
         <v>8</v>
       </c>
       <c r="E225" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -5133,11 +5133,11 @@
         <v>8</v>
       </c>
       <c r="E257" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -5717,11 +5717,11 @@
         <v>8</v>
       </c>
       <c r="E289" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -6301,11 +6301,11 @@
         <v>8</v>
       </c>
       <c r="E321" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -6885,11 +6885,11 @@
         <v>8</v>
       </c>
       <c r="E353" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -7469,11 +7469,11 @@
         <v>8</v>
       </c>
       <c r="E385" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -8053,11 +8053,11 @@
         <v>8</v>
       </c>
       <c r="E417" t="n">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -8637,11 +8637,11 @@
         <v>8</v>
       </c>
       <c r="E449" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -9221,11 +9221,11 @@
         <v>8</v>
       </c>
       <c r="E481" t="n">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="F481" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -9805,11 +9805,11 @@
         <v>8</v>
       </c>
       <c r="E513" t="n">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="F513" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -10389,11 +10389,11 @@
         <v>8</v>
       </c>
       <c r="E545" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -10973,11 +10973,11 @@
         <v>8</v>
       </c>
       <c r="E577" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="F577" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -11557,11 +11557,11 @@
         <v>8</v>
       </c>
       <c r="E609" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F609" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -12141,11 +12141,11 @@
         <v>8</v>
       </c>
       <c r="E641" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -12725,11 +12725,11 @@
         <v>8</v>
       </c>
       <c r="E673" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F673" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -13309,11 +13309,11 @@
         <v>8</v>
       </c>
       <c r="E705" t="n">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="F705" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -13893,11 +13893,11 @@
         <v>8</v>
       </c>
       <c r="E737" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F737" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -14477,11 +14477,11 @@
         <v>8</v>
       </c>
       <c r="E769" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F769" t="inlineStr">
         <is>
-          <t>2026-08-11 07:43</t>
+          <t>2026-08-12 07:51</t>
         </is>
       </c>
     </row>
@@ -14801,7 +14801,7 @@
         <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>365</v>
+        <v>399</v>
       </c>
     </row>
     <row r="3">
@@ -14904,7 +14904,7 @@
         <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>406</v>
+        <v>453</v>
       </c>
     </row>
     <row r="4">
@@ -15007,7 +15007,7 @@
         <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>308</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5">
@@ -15110,7 +15110,7 @@
         <v>0</v>
       </c>
       <c r="AG5" t="n">
-        <v>322</v>
+        <v>350</v>
       </c>
     </row>
     <row r="6">
@@ -15213,7 +15213,7 @@
         <v>4326</v>
       </c>
       <c r="AG6" t="n">
-        <v>1401</v>
+        <v>1534</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-08-18 10:21 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1045,11 +1045,11 @@
         <v>8</v>
       </c>
       <c r="E33" t="n">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -1629,11 +1629,11 @@
         <v>8</v>
       </c>
       <c r="E65" t="n">
-        <v>263</v>
+        <v>290</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -2213,11 +2213,11 @@
         <v>8</v>
       </c>
       <c r="E97" t="n">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -3381,11 +3381,11 @@
         <v>8</v>
       </c>
       <c r="E161" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -3965,11 +3965,11 @@
         <v>8</v>
       </c>
       <c r="E193" t="n">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -4549,11 +4549,11 @@
         <v>8</v>
       </c>
       <c r="E225" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -5133,11 +5133,11 @@
         <v>8</v>
       </c>
       <c r="E257" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -5717,11 +5717,11 @@
         <v>8</v>
       </c>
       <c r="E289" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -6301,11 +6301,11 @@
         <v>8</v>
       </c>
       <c r="E321" t="n">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -6885,11 +6885,11 @@
         <v>8</v>
       </c>
       <c r="E353" t="n">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -7469,11 +7469,11 @@
         <v>8</v>
       </c>
       <c r="E385" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -8053,11 +8053,11 @@
         <v>8</v>
       </c>
       <c r="E417" t="n">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -8637,11 +8637,11 @@
         <v>8</v>
       </c>
       <c r="E449" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -9221,11 +9221,11 @@
         <v>8</v>
       </c>
       <c r="E481" t="n">
-        <v>237</v>
+        <v>252</v>
       </c>
       <c r="F481" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -9805,11 +9805,11 @@
         <v>8</v>
       </c>
       <c r="E513" t="n">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="F513" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -10389,11 +10389,11 @@
         <v>8</v>
       </c>
       <c r="E545" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -10973,11 +10973,11 @@
         <v>8</v>
       </c>
       <c r="E577" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="F577" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -11557,11 +11557,11 @@
         <v>8</v>
       </c>
       <c r="E609" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="F609" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -12141,11 +12141,11 @@
         <v>8</v>
       </c>
       <c r="E641" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -12725,11 +12725,11 @@
         <v>8</v>
       </c>
       <c r="E673" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F673" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -13309,11 +13309,11 @@
         <v>8</v>
       </c>
       <c r="E705" t="n">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="F705" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -13893,11 +13893,11 @@
         <v>8</v>
       </c>
       <c r="E737" t="n">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="F737" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -14477,11 +14477,11 @@
         <v>8</v>
       </c>
       <c r="E769" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F769" t="inlineStr">
         <is>
-          <t>2026-08-17 07:21</t>
+          <t>2026-08-18 07:18</t>
         </is>
       </c>
     </row>
@@ -14801,7 +14801,7 @@
         <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>557</v>
+        <v>614</v>
       </c>
     </row>
     <row r="3">
@@ -14904,7 +14904,7 @@
         <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>653</v>
+        <v>716</v>
       </c>
     </row>
     <row r="4">
@@ -15007,7 +15007,7 @@
         <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>440</v>
+        <v>483</v>
       </c>
     </row>
     <row r="5">
@@ -15110,7 +15110,7 @@
         <v>0</v>
       </c>
       <c r="AG5" t="n">
-        <v>515</v>
+        <v>561</v>
       </c>
     </row>
     <row r="6">
@@ -15213,7 +15213,7 @@
         <v>4326</v>
       </c>
       <c r="AG6" t="n">
-        <v>2165</v>
+        <v>2374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-08-19 10:26 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1045,11 +1045,11 @@
         <v>8</v>
       </c>
       <c r="E33" t="n">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -1629,11 +1629,11 @@
         <v>8</v>
       </c>
       <c r="E65" t="n">
-        <v>290</v>
+        <v>308</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -2213,11 +2213,11 @@
         <v>8</v>
       </c>
       <c r="E97" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -3381,11 +3381,11 @@
         <v>8</v>
       </c>
       <c r="E161" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -3965,11 +3965,11 @@
         <v>8</v>
       </c>
       <c r="E193" t="n">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -4549,11 +4549,11 @@
         <v>8</v>
       </c>
       <c r="E225" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -5133,11 +5133,11 @@
         <v>8</v>
       </c>
       <c r="E257" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -5717,11 +5717,11 @@
         <v>8</v>
       </c>
       <c r="E289" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -6301,11 +6301,11 @@
         <v>8</v>
       </c>
       <c r="E321" t="n">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -6885,11 +6885,11 @@
         <v>8</v>
       </c>
       <c r="E353" t="n">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -7469,11 +7469,11 @@
         <v>8</v>
       </c>
       <c r="E385" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -8053,11 +8053,11 @@
         <v>8</v>
       </c>
       <c r="E417" t="n">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -8637,11 +8637,11 @@
         <v>8</v>
       </c>
       <c r="E449" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -9221,11 +9221,11 @@
         <v>8</v>
       </c>
       <c r="E481" t="n">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="F481" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -9805,11 +9805,11 @@
         <v>8</v>
       </c>
       <c r="E513" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="F513" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -10393,7 +10393,7 @@
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -10973,11 +10973,11 @@
         <v>8</v>
       </c>
       <c r="E577" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="F577" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -11557,11 +11557,11 @@
         <v>8</v>
       </c>
       <c r="E609" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F609" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -12141,11 +12141,11 @@
         <v>8</v>
       </c>
       <c r="E641" t="n">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -12725,11 +12725,11 @@
         <v>8</v>
       </c>
       <c r="E673" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F673" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -13309,11 +13309,11 @@
         <v>8</v>
       </c>
       <c r="E705" t="n">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="F705" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -13893,11 +13893,11 @@
         <v>8</v>
       </c>
       <c r="E737" t="n">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="F737" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -14477,11 +14477,11 @@
         <v>8</v>
       </c>
       <c r="E769" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F769" t="inlineStr">
         <is>
-          <t>2026-08-18 07:18</t>
+          <t>2026-08-19 07:23</t>
         </is>
       </c>
     </row>
@@ -14801,7 +14801,7 @@
         <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>614</v>
+        <v>650</v>
       </c>
     </row>
     <row r="3">
@@ -14904,7 +14904,7 @@
         <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>716</v>
+        <v>772</v>
       </c>
     </row>
     <row r="4">
@@ -15007,7 +15007,7 @@
         <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>483</v>
+        <v>510</v>
       </c>
     </row>
     <row r="5">
@@ -15110,7 +15110,7 @@
         <v>0</v>
       </c>
       <c r="AG5" t="n">
-        <v>561</v>
+        <v>595</v>
       </c>
     </row>
     <row r="6">
@@ -15213,7 +15213,7 @@
         <v>4326</v>
       </c>
       <c r="AG6" t="n">
-        <v>2374</v>
+        <v>2527</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-08-20 10:22 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1045,11 +1045,11 @@
         <v>8</v>
       </c>
       <c r="E33" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -1629,11 +1629,11 @@
         <v>8</v>
       </c>
       <c r="E65" t="n">
-        <v>308</v>
+        <v>337</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -2213,11 +2213,11 @@
         <v>8</v>
       </c>
       <c r="E97" t="n">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -3381,11 +3381,11 @@
         <v>8</v>
       </c>
       <c r="E161" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -3965,11 +3965,11 @@
         <v>8</v>
       </c>
       <c r="E193" t="n">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -4549,11 +4549,11 @@
         <v>8</v>
       </c>
       <c r="E225" t="n">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -5133,11 +5133,11 @@
         <v>8</v>
       </c>
       <c r="E257" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -5717,11 +5717,11 @@
         <v>8</v>
       </c>
       <c r="E289" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -6301,11 +6301,11 @@
         <v>8</v>
       </c>
       <c r="E321" t="n">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -6885,11 +6885,11 @@
         <v>8</v>
       </c>
       <c r="E353" t="n">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -7469,11 +7469,11 @@
         <v>8</v>
       </c>
       <c r="E385" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -8053,11 +8053,11 @@
         <v>8</v>
       </c>
       <c r="E417" t="n">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -8637,11 +8637,11 @@
         <v>8</v>
       </c>
       <c r="E449" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -9221,11 +9221,11 @@
         <v>8</v>
       </c>
       <c r="E481" t="n">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="F481" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -9805,11 +9805,11 @@
         <v>8</v>
       </c>
       <c r="E513" t="n">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="F513" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -10389,11 +10389,11 @@
         <v>8</v>
       </c>
       <c r="E545" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -10973,11 +10973,11 @@
         <v>8</v>
       </c>
       <c r="E577" t="n">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F577" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -11561,7 +11561,7 @@
       </c>
       <c r="F609" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -12141,11 +12141,11 @@
         <v>8</v>
       </c>
       <c r="E641" t="n">
-        <v>127</v>
+        <v>147</v>
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -12725,11 +12725,11 @@
         <v>8</v>
       </c>
       <c r="E673" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F673" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -13309,11 +13309,11 @@
         <v>8</v>
       </c>
       <c r="E705" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F705" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -13893,11 +13893,11 @@
         <v>8</v>
       </c>
       <c r="E737" t="n">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="F737" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -14477,11 +14477,11 @@
         <v>8</v>
       </c>
       <c r="E769" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F769" t="inlineStr">
         <is>
-          <t>2026-08-19 07:23</t>
+          <t>2026-08-20 07:19</t>
         </is>
       </c>
     </row>
@@ -14801,7 +14801,7 @@
         <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>650</v>
+        <v>690</v>
       </c>
     </row>
     <row r="3">
@@ -14904,7 +14904,7 @@
         <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>772</v>
+        <v>829</v>
       </c>
     </row>
     <row r="4">
@@ -15007,7 +15007,7 @@
         <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>510</v>
+        <v>543</v>
       </c>
     </row>
     <row r="5">
@@ -15110,7 +15110,7 @@
         <v>0</v>
       </c>
       <c r="AG5" t="n">
-        <v>595</v>
+        <v>635</v>
       </c>
     </row>
     <row r="6">
@@ -15213,7 +15213,7 @@
         <v>4326</v>
       </c>
       <c r="AG6" t="n">
-        <v>2527</v>
+        <v>2697</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-08-26 10:29 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1045,11 +1045,11 @@
         <v>8</v>
       </c>
       <c r="E33" t="n">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -1629,11 +1629,11 @@
         <v>8</v>
       </c>
       <c r="E65" t="n">
-        <v>439</v>
+        <v>463</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -2213,11 +2213,11 @@
         <v>8</v>
       </c>
       <c r="E97" t="n">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -3381,11 +3381,11 @@
         <v>8</v>
       </c>
       <c r="E161" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -3965,11 +3965,11 @@
         <v>8</v>
       </c>
       <c r="E193" t="n">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -4549,11 +4549,11 @@
         <v>8</v>
       </c>
       <c r="E225" t="n">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -5133,11 +5133,11 @@
         <v>8</v>
       </c>
       <c r="E257" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -5717,11 +5717,11 @@
         <v>8</v>
       </c>
       <c r="E289" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -6301,11 +6301,11 @@
         <v>8</v>
       </c>
       <c r="E321" t="n">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -6885,11 +6885,11 @@
         <v>8</v>
       </c>
       <c r="E353" t="n">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -7469,11 +7469,11 @@
         <v>8</v>
       </c>
       <c r="E385" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -8053,11 +8053,11 @@
         <v>8</v>
       </c>
       <c r="E417" t="n">
-        <v>213</v>
+        <v>224</v>
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -8637,11 +8637,11 @@
         <v>8</v>
       </c>
       <c r="E449" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -9221,11 +9221,11 @@
         <v>8</v>
       </c>
       <c r="E481" t="n">
-        <v>370</v>
+        <v>383</v>
       </c>
       <c r="F481" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -9805,11 +9805,11 @@
         <v>8</v>
       </c>
       <c r="E513" t="n">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="F513" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -10389,11 +10389,11 @@
         <v>8</v>
       </c>
       <c r="E545" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -10973,11 +10973,11 @@
         <v>8</v>
       </c>
       <c r="E577" t="n">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="F577" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -11557,11 +11557,11 @@
         <v>8</v>
       </c>
       <c r="E609" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F609" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -12141,11 +12141,11 @@
         <v>8</v>
       </c>
       <c r="E641" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -12725,11 +12725,11 @@
         <v>8</v>
       </c>
       <c r="E673" t="n">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="F673" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -13309,11 +13309,11 @@
         <v>8</v>
       </c>
       <c r="E705" t="n">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="F705" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -13893,11 +13893,11 @@
         <v>8</v>
       </c>
       <c r="E737" t="n">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="F737" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -14481,7 +14481,7 @@
       </c>
       <c r="F769" t="inlineStr">
         <is>
-          <t>2026-08-25 07:23</t>
+          <t>2026-08-26 07:25</t>
         </is>
       </c>
     </row>
@@ -14801,7 +14801,7 @@
         <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>868</v>
+        <v>904</v>
       </c>
     </row>
     <row r="3">
@@ -14904,7 +14904,7 @@
         <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>1036</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="4">
@@ -15007,7 +15007,7 @@
         <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>637</v>
+        <v>675</v>
       </c>
     </row>
     <row r="5">
@@ -15110,7 +15110,7 @@
         <v>0</v>
       </c>
       <c r="AG5" t="n">
-        <v>853</v>
+        <v>890</v>
       </c>
     </row>
     <row r="6">
@@ -15213,7 +15213,7 @@
         <v>4326</v>
       </c>
       <c r="AG6" t="n">
-        <v>3394</v>
+        <v>3561</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-08-28 21:06 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1045,11 +1045,11 @@
         <v>8</v>
       </c>
       <c r="E33" t="n">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -1629,11 +1629,11 @@
         <v>8</v>
       </c>
       <c r="E65" t="n">
-        <v>493</v>
+        <v>506</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -2213,11 +2213,11 @@
         <v>8</v>
       </c>
       <c r="E97" t="n">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -3381,11 +3381,11 @@
         <v>8</v>
       </c>
       <c r="E161" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -3965,11 +3965,11 @@
         <v>8</v>
       </c>
       <c r="E193" t="n">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -4549,11 +4549,11 @@
         <v>8</v>
       </c>
       <c r="E225" t="n">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -5133,11 +5133,11 @@
         <v>8</v>
       </c>
       <c r="E257" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -5717,11 +5717,11 @@
         <v>8</v>
       </c>
       <c r="E289" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -6301,11 +6301,11 @@
         <v>8</v>
       </c>
       <c r="E321" t="n">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -6885,11 +6885,11 @@
         <v>8</v>
       </c>
       <c r="E353" t="n">
-        <v>240</v>
+        <v>253</v>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -7469,11 +7469,11 @@
         <v>8</v>
       </c>
       <c r="E385" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -8053,11 +8053,11 @@
         <v>8</v>
       </c>
       <c r="E417" t="n">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -8637,11 +8637,11 @@
         <v>8</v>
       </c>
       <c r="E449" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -9221,11 +9221,11 @@
         <v>8</v>
       </c>
       <c r="E481" t="n">
-        <v>415</v>
+        <v>437</v>
       </c>
       <c r="F481" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -9805,11 +9805,11 @@
         <v>8</v>
       </c>
       <c r="E513" t="n">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="F513" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -10393,7 +10393,7 @@
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -10973,11 +10973,11 @@
         <v>8</v>
       </c>
       <c r="E577" t="n">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F577" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -11557,11 +11557,11 @@
         <v>8</v>
       </c>
       <c r="E609" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F609" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -12141,11 +12141,11 @@
         <v>8</v>
       </c>
       <c r="E641" t="n">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -12725,11 +12725,11 @@
         <v>8</v>
       </c>
       <c r="E673" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F673" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -13309,11 +13309,11 @@
         <v>8</v>
       </c>
       <c r="E705" t="n">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="F705" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -13893,11 +13893,11 @@
         <v>8</v>
       </c>
       <c r="E737" t="n">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="F737" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -14477,11 +14477,11 @@
         <v>8</v>
       </c>
       <c r="E769" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="F769" t="inlineStr">
         <is>
-          <t>2026-08-27 17:06</t>
+          <t>2026-08-28 18:03</t>
         </is>
       </c>
     </row>
@@ -14801,7 +14801,7 @@
         <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>952</v>
+        <v>986</v>
       </c>
     </row>
     <row r="3">
@@ -14904,7 +14904,7 @@
         <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>1152</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="4">
@@ -15007,7 +15007,7 @@
         <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>729</v>
+        <v>767</v>
       </c>
     </row>
     <row r="5">
@@ -15110,7 +15110,7 @@
         <v>0</v>
       </c>
       <c r="AG5" t="n">
-        <v>956</v>
+        <v>997</v>
       </c>
     </row>
     <row r="6">
@@ -15213,7 +15213,7 @@
         <v>4326</v>
       </c>
       <c r="AG6" t="n">
-        <v>3789</v>
+        <v>3942</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-08-31 17:21 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1045,11 +1045,11 @@
         <v>8</v>
       </c>
       <c r="E33" t="n">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -1629,11 +1629,11 @@
         <v>8</v>
       </c>
       <c r="E65" t="n">
-        <v>540</v>
+        <v>560</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -2213,11 +2213,11 @@
         <v>8</v>
       </c>
       <c r="E97" t="n">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -3381,11 +3381,11 @@
         <v>8</v>
       </c>
       <c r="E161" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -3965,11 +3965,11 @@
         <v>8</v>
       </c>
       <c r="E193" t="n">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -4549,11 +4549,11 @@
         <v>8</v>
       </c>
       <c r="E225" t="n">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -5133,11 +5133,11 @@
         <v>8</v>
       </c>
       <c r="E257" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -5717,11 +5717,11 @@
         <v>8</v>
       </c>
       <c r="E289" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -6301,11 +6301,11 @@
         <v>8</v>
       </c>
       <c r="E321" t="n">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -6885,11 +6885,11 @@
         <v>8</v>
       </c>
       <c r="E353" t="n">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -7469,11 +7469,11 @@
         <v>8</v>
       </c>
       <c r="E385" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -8053,11 +8053,11 @@
         <v>8</v>
       </c>
       <c r="E417" t="n">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -8637,11 +8637,11 @@
         <v>8</v>
       </c>
       <c r="E449" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -9221,11 +9221,11 @@
         <v>8</v>
       </c>
       <c r="E481" t="n">
-        <v>461</v>
+        <v>478</v>
       </c>
       <c r="F481" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -9805,11 +9805,11 @@
         <v>8</v>
       </c>
       <c r="E513" t="n">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="F513" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -10389,11 +10389,11 @@
         <v>8</v>
       </c>
       <c r="E545" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -10973,11 +10973,11 @@
         <v>8</v>
       </c>
       <c r="E577" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F577" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -11557,11 +11557,11 @@
         <v>8</v>
       </c>
       <c r="E609" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="F609" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -12141,11 +12141,11 @@
         <v>8</v>
       </c>
       <c r="E641" t="n">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -12725,11 +12725,11 @@
         <v>8</v>
       </c>
       <c r="E673" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="F673" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -13309,11 +13309,11 @@
         <v>8</v>
       </c>
       <c r="E705" t="n">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="F705" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -13893,11 +13893,11 @@
         <v>8</v>
       </c>
       <c r="E737" t="n">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="F737" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -14477,11 +14477,11 @@
         <v>8</v>
       </c>
       <c r="E769" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F769" t="inlineStr">
         <is>
-          <t>2026-08-30 11:36</t>
+          <t>2026-08-31 14:17</t>
         </is>
       </c>
     </row>
@@ -14801,7 +14801,7 @@
         <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>1024</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="3">
@@ -14904,7 +14904,7 @@
         <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>1230</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="4">
@@ -15007,7 +15007,7 @@
         <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>798</v>
+        <v>820</v>
       </c>
     </row>
     <row r="5">
@@ -15110,7 +15110,7 @@
         <v>0</v>
       </c>
       <c r="AG5" t="n">
-        <v>1059</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="6">
@@ -15213,7 +15213,7 @@
         <v>4326</v>
       </c>
       <c r="AG6" t="n">
-        <v>4111</v>
+        <v>4248</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-09-02 13:58 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1063,11 +1063,11 @@
         <v>9</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -1665,11 +1665,11 @@
         <v>9</v>
       </c>
       <c r="E67" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -2267,11 +2267,11 @@
         <v>9</v>
       </c>
       <c r="E100" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -3471,11 +3471,11 @@
         <v>9</v>
       </c>
       <c r="E166" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -4073,11 +4073,11 @@
         <v>9</v>
       </c>
       <c r="E199" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -4675,11 +4675,11 @@
         <v>9</v>
       </c>
       <c r="E232" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -5277,11 +5277,11 @@
         <v>9</v>
       </c>
       <c r="E265" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -5879,11 +5879,11 @@
         <v>9</v>
       </c>
       <c r="E298" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -6481,11 +6481,11 @@
         <v>9</v>
       </c>
       <c r="E331" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -7083,11 +7083,11 @@
         <v>9</v>
       </c>
       <c r="E364" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -7685,11 +7685,11 @@
         <v>9</v>
       </c>
       <c r="E397" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -8287,11 +8287,11 @@
         <v>9</v>
       </c>
       <c r="E430" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -8889,11 +8889,11 @@
         <v>9</v>
       </c>
       <c r="E463" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -9491,11 +9491,11 @@
         <v>9</v>
       </c>
       <c r="E496" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F496" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -10093,11 +10093,11 @@
         <v>9</v>
       </c>
       <c r="E529" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F529" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -10695,11 +10695,11 @@
         <v>9</v>
       </c>
       <c r="E562" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F562" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -11297,11 +11297,11 @@
         <v>9</v>
       </c>
       <c r="E595" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F595" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -11903,7 +11903,7 @@
       </c>
       <c r="F628" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -12501,11 +12501,11 @@
         <v>9</v>
       </c>
       <c r="E661" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="F661" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -13103,11 +13103,11 @@
         <v>9</v>
       </c>
       <c r="E694" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F694" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -13705,11 +13705,11 @@
         <v>9</v>
       </c>
       <c r="E727" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="F727" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -14307,11 +14307,11 @@
         <v>9</v>
       </c>
       <c r="E760" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F760" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -14909,11 +14909,11 @@
         <v>9</v>
       </c>
       <c r="E793" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F793" t="inlineStr">
         <is>
-          <t>2026-09-01 11:21</t>
+          <t>2026-09-02 10:56</t>
         </is>
       </c>
     </row>
@@ -15242,7 +15242,7 @@
         <v>0</v>
       </c>
       <c r="AH2" t="n">
-        <v>11</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3">
@@ -15348,7 +15348,7 @@
         <v>0</v>
       </c>
       <c r="AH3" t="n">
-        <v>13</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4">
@@ -15454,7 +15454,7 @@
         <v>0</v>
       </c>
       <c r="AH4" t="n">
-        <v>12</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5">
@@ -15560,7 +15560,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="n">
-        <v>17</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6">
@@ -15666,7 +15666,7 @@
         <v>4248</v>
       </c>
       <c r="AH6" t="n">
-        <v>53</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard: 2026-09-03 14:00 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/historico_leads.xlsx
+++ b/greenlife_scraper/historico_leads.xlsx
@@ -1063,11 +1063,11 @@
         <v>9</v>
       </c>
       <c r="E34" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -1665,11 +1665,11 @@
         <v>9</v>
       </c>
       <c r="E67" t="n">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -2267,11 +2267,11 @@
         <v>9</v>
       </c>
       <c r="E100" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -3471,11 +3471,11 @@
         <v>9</v>
       </c>
       <c r="E166" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -4073,11 +4073,11 @@
         <v>9</v>
       </c>
       <c r="E199" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -4675,11 +4675,11 @@
         <v>9</v>
       </c>
       <c r="E232" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -5277,11 +5277,11 @@
         <v>9</v>
       </c>
       <c r="E265" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -5879,11 +5879,11 @@
         <v>9</v>
       </c>
       <c r="E298" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -6481,11 +6481,11 @@
         <v>9</v>
       </c>
       <c r="E331" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -7083,11 +7083,11 @@
         <v>9</v>
       </c>
       <c r="E364" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -7689,7 +7689,7 @@
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -8287,11 +8287,11 @@
         <v>9</v>
       </c>
       <c r="E430" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -8889,11 +8889,11 @@
         <v>9</v>
       </c>
       <c r="E463" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -9491,11 +9491,11 @@
         <v>9</v>
       </c>
       <c r="E496" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F496" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -10093,11 +10093,11 @@
         <v>9</v>
       </c>
       <c r="E529" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F529" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -10695,11 +10695,11 @@
         <v>9</v>
       </c>
       <c r="E562" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F562" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -11297,11 +11297,11 @@
         <v>9</v>
       </c>
       <c r="E595" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F595" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -11899,11 +11899,11 @@
         <v>9</v>
       </c>
       <c r="E628" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F628" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -12501,11 +12501,11 @@
         <v>9</v>
       </c>
       <c r="E661" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F661" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -13103,11 +13103,11 @@
         <v>9</v>
       </c>
       <c r="E694" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F694" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -13705,11 +13705,11 @@
         <v>9</v>
       </c>
       <c r="E727" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F727" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -14307,11 +14307,11 @@
         <v>9</v>
       </c>
       <c r="E760" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F760" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -14909,11 +14909,11 @@
         <v>9</v>
       </c>
       <c r="E793" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F793" t="inlineStr">
         <is>
-          <t>2026-09-02 10:56</t>
+          <t>2026-09-03 10:58</t>
         </is>
       </c>
     </row>
@@ -15242,7 +15242,7 @@
         <v>0</v>
       </c>
       <c r="AH2" t="n">
-        <v>54</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3">
@@ -15348,7 +15348,7 @@
         <v>0</v>
       </c>
       <c r="AH3" t="n">
-        <v>69</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4">
@@ -15454,7 +15454,7 @@
         <v>0</v>
       </c>
       <c r="AH4" t="n">
-        <v>52</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5">
@@ -15560,7 +15560,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="n">
-        <v>46</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6">
@@ -15666,7 +15666,7 @@
         <v>4248</v>
       </c>
       <c r="AH6" t="n">
-        <v>221</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>